<commit_message>
Rewrite planning answer keys and fix reviewed answers
- Planning answers for all 15 planning questions now follow the
  numbered mark-scheme style (set-up, 8 readings, control of
  variables, preliminary readings, graphs that test the relationship,
  precautions, safety). They live in content/plans.py and are laid
  onto the papers with a new Paper.flow helper.
- tools/plans_pdf.py compiles every planning question with its
  answer key into one PDF (built locally; the school pages stay
  out of the repo).
- Fixes from a full review of the other answers: half-up rounding of
  T values, values that disagreed with their own working, ACJC Q2
  regenerated for the 1.5 V supply, ASRJC line W drawn, k = 4ρ/π in
  VJC/TJC, overlapping text, workbook number formats and a VJC
  workbook strip bug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014pdGBji7p4GhAVY9SYPUSG
</commit_message>
<xml_diff>
--- a/virtual-physics-lab/app/dl/ACJC_Q1_V_pendulum.xlsx
+++ b/virtual-physics-lab/app/dl/ACJC_Q1_V_pendulum.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -91,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -100,6 +102,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -692,103 +696,103 @@
       <c r="A6" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="7" t="n">
         <v>24.69</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="7" t="n">
         <v>24.77</v>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="7" t="n">
         <v>24.3</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="7" t="n">
         <v>24.08</v>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="7" t="n">
         <v>23.43</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="7" t="n">
         <v>23.51</v>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="7" t="n">
         <v>22.55</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="7" t="n">
         <v>22.53</v>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
         <v>131</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="7" t="n">
         <v>21.36</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="7" t="n">
         <v>21.28</v>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="7" t="n">
         <v>20.12</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="7" t="n">
         <v>20.18</v>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -886,24 +890,24 @@
       <c r="A6" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="7" t="n">
         <v>24.69</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="7" t="n">
         <v>24.77</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <f>(C6+D6)/40</f>
         <v/>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <f>COS(RADIANS(A6)/2)</f>
         <v/>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <f>E6^2</f>
         <v/>
       </c>
@@ -912,7 +916,7 @@
           <t>gradient = 4π²l/g</t>
         </is>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="9">
         <f>SLOPE(G6:G11,F6:F11)</f>
         <v/>
       </c>
@@ -926,24 +930,24 @@
       <c r="A7" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="7" t="n">
         <v>24.3</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="7" t="n">
         <v>24.08</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <f>(C7+D7)/40</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="9">
         <f>COS(RADIANS(A7)/2)</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <f>E7^2</f>
         <v/>
       </c>
@@ -952,7 +956,7 @@
           <t>c = intercept</t>
         </is>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="9">
         <f>INTERCEPT(G6:G11,F6:F11)</f>
         <v/>
       </c>
@@ -966,24 +970,24 @@
       <c r="A8" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="7" t="n">
         <v>23.43</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="7" t="n">
         <v>23.51</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <f>(C8+D8)/40</f>
         <v/>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="9">
         <f>COS(RADIANS(A8)/2)</f>
         <v/>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <f>E8^2</f>
         <v/>
       </c>
@@ -992,7 +996,7 @@
           <t>g = 4π²(0.200)/gradient</t>
         </is>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <f>4*PI()^2*0.2/SLOPE(G6:G11,F6:F11)</f>
         <v/>
       </c>
@@ -1006,24 +1010,24 @@
       <c r="A9" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="7" t="n">
         <v>22.55</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="7" t="n">
         <v>22.53</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <f>(C9+D9)/40</f>
         <v/>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="9">
         <f>COS(RADIANS(A9)/2)</f>
         <v/>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="9">
         <f>E9^2</f>
         <v/>
       </c>
@@ -1032,24 +1036,24 @@
       <c r="A10" s="5" t="n">
         <v>131</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="7" t="n">
         <v>21.36</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="7" t="n">
         <v>21.28</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="9">
         <f>(C10+D10)/40</f>
         <v/>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="9">
         <f>COS(RADIANS(A10)/2)</f>
         <v/>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="9">
         <f>E10^2</f>
         <v/>
       </c>
@@ -1058,24 +1062,24 @@
       <c r="A11" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="7" t="n">
         <v>20.12</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="7" t="n">
         <v>20.18</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="9">
         <f>(C11+D11)/40</f>
         <v/>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="9">
         <f>COS(RADIANS(A11)/2)</f>
         <v/>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="9">
         <f>E11^2</f>
         <v/>
       </c>

</xml_diff>